<commit_message>
add function to identify bad X-ray entries not present in CWL; update outputs and weights
</commit_message>
<xml_diff>
--- a/inputs/cwl-responses.xlsx
+++ b/inputs/cwl-responses.xlsx
@@ -6,14 +6,14 @@
     <sheet state="visible" name="Form Responses 1" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Form Responses 1'!$A$1:$E$38</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Form Responses 1'!$A$1:$E$39</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="59">
   <si>
     <t>Timestamp</t>
   </si>
@@ -42,6 +42,9 @@
     <t>¯\_(ツ)_/¯</t>
   </si>
   <si>
+    <t>Ratchet</t>
+  </si>
+  <si>
     <t>Sned</t>
   </si>
   <si>
@@ -54,7 +57,7 @@
     <t>Dr. Stone</t>
   </si>
   <si>
-    <t>Satan</t>
+    <t>God Sukuna</t>
   </si>
   <si>
     <t>All 7 wars</t>
@@ -63,12 +66,6 @@
     <t>Vojt</t>
   </si>
   <si>
-    <t>Erdnussflip</t>
-  </si>
-  <si>
-    <t>Yo</t>
-  </si>
-  <si>
     <t>osiris8282</t>
   </si>
   <si>
@@ -102,12 +99,21 @@
     <t>RoyalOne</t>
   </si>
   <si>
+    <t>S4VAGE_B5</t>
+  </si>
+  <si>
+    <t>LET'S GET IT!!</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ascended </t>
   </si>
   <si>
     <t>GLHF</t>
   </si>
   <si>
+    <t>DNG</t>
+  </si>
+  <si>
     <t>ÍâmGrøØt</t>
   </si>
   <si>
@@ -117,18 +123,9 @@
     <t>Nope</t>
   </si>
   <si>
-    <t>S4VAGE_B5</t>
-  </si>
-  <si>
-    <t>LET'S GO!!!</t>
-  </si>
-  <si>
     <t>⚡TANJIRO⚡</t>
   </si>
   <si>
-    <t>DNG</t>
-  </si>
-  <si>
     <t>Rod</t>
   </si>
   <si>
@@ -171,10 +168,16 @@
     <t>busy with uni :/</t>
   </si>
   <si>
+    <t>beeche</t>
+  </si>
+  <si>
+    <t>Standby / bench</t>
+  </si>
+  <si>
+    <t>loveya</t>
+  </si>
+  <si>
     <t>Hype</t>
-  </si>
-  <si>
-    <t>Standby / bench</t>
   </si>
   <si>
     <t>your mama</t>
@@ -567,7 +570,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2">
-        <v>45992.53903111111</v>
+        <v>46142.56484590277</v>
       </c>
       <c r="B4" s="3">
         <v>18.0</v>
@@ -582,10 +585,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2">
-        <v>46114.732371562495</v>
+        <v>45992.53903111111</v>
       </c>
       <c r="B5" s="3">
-        <v>15.0</v>
+        <v>18.0</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>10</v>
@@ -597,10 +600,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2">
-        <v>45992.51229436343</v>
+        <v>46114.732371562495</v>
       </c>
       <c r="B6" s="3">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>11</v>
@@ -612,10 +615,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2">
-        <v>46054.83765527778</v>
+        <v>45992.51229436343</v>
       </c>
       <c r="B7" s="3">
-        <v>13.0</v>
+        <v>14.0</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>12</v>
@@ -627,50 +630,48 @@
     </row>
     <row r="8">
       <c r="A8" s="2">
-        <v>45994.4538564699</v>
+        <v>46054.83765527778</v>
       </c>
       <c r="B8" s="3">
-        <v>18.0</v>
+        <v>13.0</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E8" s="4"/>
     </row>
     <row r="9">
       <c r="A9" s="2">
-        <v>45648.90493895834</v>
+        <v>46143.37103672454</v>
       </c>
       <c r="B9" s="3">
         <v>18.0</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E9" s="4"/>
     </row>
     <row r="10">
       <c r="A10" s="2">
-        <v>45993.1042916088</v>
+        <v>45648.90493895834</v>
       </c>
       <c r="B10" s="3">
-        <v>17.0</v>
+        <v>18.0</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>17</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="E10" s="4"/>
     </row>
     <row r="11">
       <c r="A11" s="2">
@@ -680,13 +681,13 @@
         <v>17.0</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="12">
@@ -697,10 +698,10 @@
         <v>17.0</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E12" s="4"/>
     </row>
@@ -712,10 +713,10 @@
         <v>17.0</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E13" s="4"/>
     </row>
@@ -727,10 +728,10 @@
         <v>17.0</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E14" s="4"/>
     </row>
@@ -742,10 +743,10 @@
         <v>17.0</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E15" s="4"/>
     </row>
@@ -757,10 +758,10 @@
         <v>17.0</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E16" s="4"/>
     </row>
@@ -772,10 +773,10 @@
         <v>17.0</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E17" s="4"/>
     </row>
@@ -787,10 +788,10 @@
         <v>16.0</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E18" s="4"/>
     </row>
@@ -802,10 +803,10 @@
         <v>16.0</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E19" s="4"/>
     </row>
@@ -817,48 +818,50 @@
         <v>16.0</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E20" s="4"/>
     </row>
     <row r="21">
       <c r="A21" s="2">
-        <v>45679.996027534726</v>
+        <v>46142.58193027778</v>
       </c>
       <c r="B21" s="3">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
       <c r="C21" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2">
-        <v>46111.44214675926</v>
+        <v>45679.996027534726</v>
       </c>
       <c r="B22" s="3">
         <v>15.0</v>
       </c>
       <c r="C22" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E22" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D22" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E22" s="4"/>
     </row>
     <row r="23">
       <c r="A23" s="2">
-        <v>46019.079862557875</v>
+        <v>46142.08724311343</v>
       </c>
       <c r="B23" s="3">
         <v>15.0</v>
@@ -867,56 +870,54 @@
         <v>32</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>33</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="E23" s="4"/>
     </row>
     <row r="24">
       <c r="A24" s="2">
-        <v>46113.72583660879</v>
+        <v>46111.44214675926</v>
       </c>
       <c r="B24" s="3">
         <v>15.0</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>35</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="E24" s="4"/>
     </row>
     <row r="25">
       <c r="A25" s="2">
-        <v>46054.83679070602</v>
+        <v>46019.079862557875</v>
       </c>
       <c r="B25" s="3">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E25" s="4"/>
+        <v>15</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2">
-        <v>45956.92735099537</v>
+        <v>46054.83679070602</v>
       </c>
       <c r="B26" s="3">
         <v>14.0</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E26" s="4"/>
     </row>
@@ -928,13 +929,13 @@
         <v>14.0</v>
       </c>
       <c r="C27" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>38</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="28">
@@ -945,10 +946,10 @@
         <v>14.0</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E28" s="4"/>
     </row>
@@ -960,13 +961,13 @@
         <v>13.0</v>
       </c>
       <c r="C29" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E29" s="3" t="s">
         <v>41</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="30">
@@ -977,13 +978,13 @@
         <v>16.0</v>
       </c>
       <c r="C30" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D30" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="E30" s="3" t="s">
         <v>44</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="31">
@@ -994,10 +995,10 @@
         <v>16.0</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E31" s="4"/>
     </row>
@@ -1009,10 +1010,10 @@
         <v>14.0</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E32" s="4"/>
     </row>
@@ -1024,13 +1025,13 @@
         <v>14.0</v>
       </c>
       <c r="C33" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="D33" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="34">
@@ -1041,102 +1042,119 @@
         <v>13.0</v>
       </c>
       <c r="C34" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E34" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2">
-        <v>46054.611736770836</v>
+        <v>46142.288890428244</v>
       </c>
       <c r="B35" s="3">
         <v>16.0</v>
       </c>
       <c r="C35" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D35" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="E35" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E35" s="4"/>
     </row>
     <row r="36">
       <c r="A36" s="2">
-        <v>45961.01037400463</v>
+        <v>46054.611736770836</v>
       </c>
       <c r="B36" s="3">
-        <v>14.0</v>
+        <v>16.0</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>54</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>55</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="E36" s="4"/>
     </row>
     <row r="37">
       <c r="A37" s="2">
-        <v>45833.69785351852</v>
+        <v>45961.01037400463</v>
       </c>
       <c r="B37" s="3">
-        <v>13.0</v>
+        <v>14.0</v>
       </c>
       <c r="C37" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E37" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D37" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="E37" s="4"/>
     </row>
     <row r="38">
       <c r="A38" s="2">
-        <v>45932.63639908565</v>
+        <v>45833.69785351852</v>
       </c>
       <c r="B38" s="3">
-        <v>12.0</v>
+        <v>13.0</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>57</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E38" s="4"/>
     </row>
     <row r="39">
-      <c r="A39" s="5"/>
-      <c r="B39" s="5"/>
-      <c r="C39" s="5"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="5"/>
+      <c r="A39" s="2">
+        <v>45932.63639908565</v>
+      </c>
+      <c r="B39" s="3">
+        <v>12.0</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E39" s="4"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5"/>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="$A$1:$E$38"/>
-  <conditionalFormatting sqref="A1:E39">
+  <autoFilter ref="$A$1:$E$39"/>
+  <conditionalFormatting sqref="A1:E40">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$D1="All 7 wars"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:E39">
+  <conditionalFormatting sqref="A1:E40">
     <cfRule type="expression" dxfId="1" priority="2">
       <formula>$D1="None (participation medals only)"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:E39">
+  <conditionalFormatting sqref="A1:E40">
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>$D1="Standby / bench"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:E39">
+  <conditionalFormatting sqref="A1:E40">
     <cfRule type="expression" dxfId="3" priority="4">
       <formula>$D1="8 stars only"</formula>
     </cfRule>

</xml_diff>